<commit_message>
apply desgin to excel tables
</commit_message>
<xml_diff>
--- a/data/outputs/2024-11-22_2024-11-26/general_statistic.xlsx
+++ b/data/outputs/2024-11-22_2024-11-26/general_statistic.xlsx
@@ -622,13 +622,13 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -753,7 +753,7 @@
         <v>-0.0636</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0.9091</v>
@@ -783,7 +783,7 @@
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>